<commit_message>
Spreadsheets: gray placeholder hints and a pop-up instruction in every input
Each empty yellow cell now shows a gray italic hint ("e.g. 250,000",
"leave if none", "choose ▾"). Hints are text, so SUM / N() / ISNUMBER
ignore them and totals stay at zero until a real number is typed; a
conditional format shows typed numbers in black. Every input has an input
message (Excel and Google Sheets) saying what to type. Money Map, Net Worth
Calculator and Goal Planner share one helper so they behave the same.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kkM6oN9Y7js9B3i7hPKTM
</commit_message>
<xml_diff>
--- a/public/magnets/goal-planner.xlsx
+++ b/public/magnets/goal-planner.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="&quot;₦&quot;#,##0;[Red]-&quot;₦&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,10 @@
     </font>
     <font>
       <color rgb="004C6A62"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="009AA8A3"/>
     </font>
     <font>
       <b val="1"/>
@@ -124,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,30 +147,49 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="00000000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -528,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B34"/>
+  <dimension ref="B1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -629,82 +652,96 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Only type in the yellow cells</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>The gray words in yellow cells are hints</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>The white cells hold formulas that do the maths. If you type over one by mistake, download a fresh copy.</t>
+          <t>Each yellow cell shows a gray hint such as "e.g. 250,000". It is only a hint: it doesn't count. Tap the cell and type your own number over it; your number turns black and the totals update. Leave the hint in any cell that doesn't apply to you. Tap a cell to see a short instruction for it.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Want to see a finished one first?</t>
+          <t>Only type in the yellow cells</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Open the "Example" tab: Esther's goals, from her emergency fund to her children's university. Don't type your own goals there.</t>
+          <t>The white cells hold formulas that do the maths. If you type over one by mistake, download a fresh copy.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>These are estimates</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="45" customHeight="1">
+          <t>Want to see a finished one first?</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The sheet assumes prices rise by the same percentage every year. Real prices don't move that neatly, which is why you check once a year. It doesn't count any interest your savings earn, so the monthly amounts are on the safe side.</t>
+          <t>Open the "Example" tab: Esther's goals, from her emergency fund to her children's university. Don't type your own goals there.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>On a phone</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
+          <t>These are estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Open the file with the free Google Sheets or Microsoft Excel app. In Google Sheets, tap File &gt; Make a copy (or Save as Google Sheets) so you can edit it and keep it.</t>
+          <t>The sheet assumes prices rise by the same percentage every year. Real prices don't move that neatly, which is why you check once a year. It doesn't count any interest your savings earn, so the monthly amounts are on the safe side.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>On a phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Open the file with the free Google Sheets or Microsoft Excel app. In Google Sheets, tap File &gt; Make a copy (or Save as Google Sheets) so you can edit it and keep it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
           <t>Your privacy</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="34" ht="15" customHeight="1">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>This file stays on your phone or computer. Nobody else sees your goals or numbers.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>From the free Financial Intelligence class: kopkad.ng/blog. For educational purposes only. This is not financial advice.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="5" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>With Snowball, we keep it rolling.</t>
         </is>
@@ -788,7 +825,11 @@
           <t>What I can save each month</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n"/>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>e.g. 160,000</t>
+        </is>
+      </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Your monthly surplus from your Money Map (money in − money out).</t>
@@ -853,310 +894,342 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="15">
-        <f>IF(E9="","",IF(F9="Yes",E9+G9,(E9*(1+$C$4)^C9+G9)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="15">
-        <f>IF(I9="","",MAX(0,I9-H9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="16">
-        <f>IF(OR(J9="",C9=""),"",IF(C9&lt;=0,J9,J9/(C9*12)))</f>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>e.g. Rent</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>choose ▾</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>e.g. 0.5</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>e.g. 1</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>e.g. 600,000</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>choose ▾</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>e.g. 0</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>e.g. 120,000</t>
+        </is>
+      </c>
+      <c r="I9" s="16">
+        <f>IF(NOT(ISNUMBER(E9)),"",IF(F9="Yes",E9+N(G9),(E9*(1+$C$4)^N(C9)+N(G9))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF(I9="","",MAX(0,I9-N(H9)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF(OR(J9="",NOT(ISNUMBER(C9))),"",IF(C9&lt;=0,J9,J9/(C9*12)))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="15">
-        <f>IF(E10="","",IF(F10="Yes",E10+G10,(E10*(1+$C$4)^C10+G10)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J10" s="15">
-        <f>IF(I10="","",MAX(0,I10-H10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="16">
-        <f>IF(OR(J10="",C10=""),"",IF(C10&lt;=0,J10,J10/(C10*12)))</f>
+      <c r="A10" s="18" t="n"/>
+      <c r="B10" s="13" t="inlineStr"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="21" t="n"/>
+      <c r="I10" s="16">
+        <f>IF(NOT(ISNUMBER(E10)),"",IF(F10="Yes",E10+N(G10),(E10*(1+$C$4)^N(C10)+N(G10))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF(I10="","",MAX(0,I10-N(H10)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF(OR(J10="",NOT(ISNUMBER(C10))),"",IF(C10&lt;=0,J10,J10/(C10*12)))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="15">
-        <f>IF(E11="","",IF(F11="Yes",E11+G11,(E11*(1+$C$4)^C11+G11)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J11" s="15">
-        <f>IF(I11="","",MAX(0,I11-H11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="16">
-        <f>IF(OR(J11="",C11=""),"",IF(C11&lt;=0,J11,J11/(C11*12)))</f>
+      <c r="A11" s="18" t="n"/>
+      <c r="B11" s="13" t="inlineStr"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="20" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="13" t="inlineStr"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="16">
+        <f>IF(NOT(ISNUMBER(E11)),"",IF(F11="Yes",E11+N(G11),(E11*(1+$C$4)^N(C11)+N(G11))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>IF(I11="","",MAX(0,I11-N(H11)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IF(OR(J11="",NOT(ISNUMBER(C11))),"",IF(C11&lt;=0,J11,J11/(C11*12)))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="15">
-        <f>IF(E12="","",IF(F12="Yes",E12+G12,(E12*(1+$C$4)^C12+G12)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J12" s="15">
-        <f>IF(I12="","",MAX(0,I12-H12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="16">
-        <f>IF(OR(J12="",C12=""),"",IF(C12&lt;=0,J12,J12/(C12*12)))</f>
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="13" t="inlineStr"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="13" t="inlineStr"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="16">
+        <f>IF(NOT(ISNUMBER(E12)),"",IF(F12="Yes",E12+N(G12),(E12*(1+$C$4)^N(C12)+N(G12))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="16">
+        <f>IF(I12="","",MAX(0,I12-N(H12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="17">
+        <f>IF(OR(J12="",NOT(ISNUMBER(C12))),"",IF(C12&lt;=0,J12,J12/(C12*12)))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
-      <c r="I13" s="15">
-        <f>IF(E13="","",IF(F13="Yes",E13+G13,(E13*(1+$C$4)^C13+G13)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J13" s="15">
-        <f>IF(I13="","",MAX(0,I13-H13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="16">
-        <f>IF(OR(J13="",C13=""),"",IF(C13&lt;=0,J13,J13/(C13*12)))</f>
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="13" t="inlineStr"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="13" t="inlineStr"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="21" t="n"/>
+      <c r="I13" s="16">
+        <f>IF(NOT(ISNUMBER(E13)),"",IF(F13="Yes",E13+N(G13),(E13*(1+$C$4)^N(C13)+N(G13))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J13" s="16">
+        <f>IF(I13="","",MAX(0,I13-N(H13)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="17">
+        <f>IF(OR(J13="",NOT(ISNUMBER(C13))),"",IF(C13&lt;=0,J13,J13/(C13*12)))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="15">
-        <f>IF(E14="","",IF(F14="Yes",E14+G14,(E14*(1+$C$4)^C14+G14)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J14" s="15">
-        <f>IF(I14="","",MAX(0,I14-H14))</f>
-        <v/>
-      </c>
-      <c r="K14" s="16">
-        <f>IF(OR(J14="",C14=""),"",IF(C14&lt;=0,J14,J14/(C14*12)))</f>
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="13" t="inlineStr"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="13" t="inlineStr"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
+      <c r="I14" s="16">
+        <f>IF(NOT(ISNUMBER(E14)),"",IF(F14="Yes",E14+N(G14),(E14*(1+$C$4)^N(C14)+N(G14))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J14" s="16">
+        <f>IF(I14="","",MAX(0,I14-N(H14)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="17">
+        <f>IF(OR(J14="",NOT(ISNUMBER(C14))),"",IF(C14&lt;=0,J14,J14/(C14*12)))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="15">
-        <f>IF(E15="","",IF(F15="Yes",E15+G15,(E15*(1+$C$4)^C15+G15)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J15" s="15">
-        <f>IF(I15="","",MAX(0,I15-H15))</f>
-        <v/>
-      </c>
-      <c r="K15" s="16">
-        <f>IF(OR(J15="",C15=""),"",IF(C15&lt;=0,J15,J15/(C15*12)))</f>
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="13" t="inlineStr"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="13" t="inlineStr"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="16">
+        <f>IF(NOT(ISNUMBER(E15)),"",IF(F15="Yes",E15+N(G15),(E15*(1+$C$4)^N(C15)+N(G15))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J15" s="16">
+        <f>IF(I15="","",MAX(0,I15-N(H15)))</f>
+        <v/>
+      </c>
+      <c r="K15" s="17">
+        <f>IF(OR(J15="",NOT(ISNUMBER(C15))),"",IF(C15&lt;=0,J15,J15/(C15*12)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="15">
-        <f>IF(E16="","",IF(F16="Yes",E16+G16,(E16*(1+$C$4)^C16+G16)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J16" s="15">
-        <f>IF(I16="","",MAX(0,I16-H16))</f>
-        <v/>
-      </c>
-      <c r="K16" s="16">
-        <f>IF(OR(J16="",C16=""),"",IF(C16&lt;=0,J16,J16/(C16*12)))</f>
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="13" t="inlineStr"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="13" t="inlineStr"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="21" t="n"/>
+      <c r="I16" s="16">
+        <f>IF(NOT(ISNUMBER(E16)),"",IF(F16="Yes",E16+N(G16),(E16*(1+$C$4)^N(C16)+N(G16))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J16" s="16">
+        <f>IF(I16="","",MAX(0,I16-N(H16)))</f>
+        <v/>
+      </c>
+      <c r="K16" s="17">
+        <f>IF(OR(J16="",NOT(ISNUMBER(C16))),"",IF(C16&lt;=0,J16,J16/(C16*12)))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="15">
-        <f>IF(E17="","",IF(F17="Yes",E17+G17,(E17*(1+$C$4)^C17+G17)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J17" s="15">
-        <f>IF(I17="","",MAX(0,I17-H17))</f>
-        <v/>
-      </c>
-      <c r="K17" s="16">
-        <f>IF(OR(J17="",C17=""),"",IF(C17&lt;=0,J17,J17/(C17*12)))</f>
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="13" t="inlineStr"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="16">
+        <f>IF(NOT(ISNUMBER(E17)),"",IF(F17="Yes",E17+N(G17),(E17*(1+$C$4)^N(C17)+N(G17))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>IF(I17="","",MAX(0,I17-N(H17)))</f>
+        <v/>
+      </c>
+      <c r="K17" s="17">
+        <f>IF(OR(J17="",NOT(ISNUMBER(C17))),"",IF(C17&lt;=0,J17,J17/(C17*12)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="15">
-        <f>IF(E18="","",IF(F18="Yes",E18+G18,(E18*(1+$C$4)^C18+G18)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J18" s="15">
-        <f>IF(I18="","",MAX(0,I18-H18))</f>
-        <v/>
-      </c>
-      <c r="K18" s="16">
-        <f>IF(OR(J18="",C18=""),"",IF(C18&lt;=0,J18,J18/(C18*12)))</f>
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="13" t="inlineStr"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="13" t="inlineStr"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="16">
+        <f>IF(NOT(ISNUMBER(E18)),"",IF(F18="Yes",E18+N(G18),(E18*(1+$C$4)^N(C18)+N(G18))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J18" s="16">
+        <f>IF(I18="","",MAX(0,I18-N(H18)))</f>
+        <v/>
+      </c>
+      <c r="K18" s="17">
+        <f>IF(OR(J18="",NOT(ISNUMBER(C18))),"",IF(C18&lt;=0,J18,J18/(C18*12)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="15">
-        <f>IF(E19="","",IF(F19="Yes",E19+G19,(E19*(1+$C$4)^C19+G19)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J19" s="15">
-        <f>IF(I19="","",MAX(0,I19-H19))</f>
-        <v/>
-      </c>
-      <c r="K19" s="16">
-        <f>IF(OR(J19="",C19=""),"",IF(C19&lt;=0,J19,J19/(C19*12)))</f>
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="13" t="inlineStr"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="13" t="inlineStr"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="16">
+        <f>IF(NOT(ISNUMBER(E19)),"",IF(F19="Yes",E19+N(G19),(E19*(1+$C$4)^N(C19)+N(G19))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>IF(I19="","",MAX(0,I19-N(H19)))</f>
+        <v/>
+      </c>
+      <c r="K19" s="17">
+        <f>IF(OR(J19="",NOT(ISNUMBER(C19))),"",IF(C19&lt;=0,J19,J19/(C19*12)))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="15">
-        <f>IF(E20="","",IF(F20="Yes",E20+G20,(E20*(1+$C$4)^C20+G20)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J20" s="15">
-        <f>IF(I20="","",MAX(0,I20-H20))</f>
-        <v/>
-      </c>
-      <c r="K20" s="16">
-        <f>IF(OR(J20="",C20=""),"",IF(C20&lt;=0,J20,J20/(C20*12)))</f>
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="13" t="inlineStr"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="13" t="inlineStr"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
+      <c r="I20" s="16">
+        <f>IF(NOT(ISNUMBER(E20)),"",IF(F20="Yes",E20+N(G20),(E20*(1+$C$4)^N(C20)+N(G20))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J20" s="16">
+        <f>IF(I20="","",MAX(0,I20-N(H20)))</f>
+        <v/>
+      </c>
+      <c r="K20" s="17">
+        <f>IF(OR(J20="",NOT(ISNUMBER(C20))),"",IF(C20&lt;=0,J20,J20/(C20*12)))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>Total needed each month for all goals</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="n"/>
-      <c r="I22" s="18" t="n"/>
-      <c r="J22" s="18" t="n"/>
-      <c r="K22" s="19">
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="23" t="n"/>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="23" t="n"/>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="23" t="n"/>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="23" t="n"/>
+      <c r="K22" s="24">
         <f>SUM(K9:K20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Can I afford all of them?</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>If "Not yet": give each goal a priority, fund the top ones first, move a date later, or start smaller.</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
-      <c r="J23" s="18" t="n"/>
-      <c r="K23" s="17">
-        <f>IF($C$6="","Fill in C6",IF(K22&lt;=$C$6,"Yes","Not yet"))</f>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="23" t="n"/>
+      <c r="J23" s="23" t="n"/>
+      <c r="K23" s="22">
+        <f>IF(NOT(ISNUMBER($C$6)),"Fill in C6",IF(K22&lt;=$C$6,"Yes","Not yet"))</f>
         <v/>
       </c>
     </row>
@@ -1168,27 +1241,663 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Free from the Financial Intelligence class · kopkad.ng/blog. For educational purposes only. This is not financial advice.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>With Snowball, we keep it rolling.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <conditionalFormatting sqref="C4">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(C4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>ISNUMBER(C5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>ISNUMBER(C6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A9">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>ISNUMBER(A9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>OR(B9="Within 1 year",B9="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>ISNUMBER(C9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>ISNUMBER(D9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>ISNUMBER(E9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>OR(F9="Yes",F9="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>ISNUMBER(G9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>ISNUMBER(H9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10">
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>ISNUMBER(A10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>OR(B10="Within 1 year",B10="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
+    <cfRule type="expression" priority="14" dxfId="0">
+      <formula>ISNUMBER(C10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>ISNUMBER(D10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>ISNUMBER(E10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F10">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>OR(F10="Yes",F10="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10">
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>ISNUMBER(G10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>ISNUMBER(H10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A11">
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>ISNUMBER(A11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>OR(B11="Within 1 year",B11="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="expression" priority="22" dxfId="0">
+      <formula>ISNUMBER(C11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11">
+    <cfRule type="expression" priority="23" dxfId="0">
+      <formula>ISNUMBER(D11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11">
+    <cfRule type="expression" priority="24" dxfId="0">
+      <formula>ISNUMBER(E11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>OR(F11="Yes",F11="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11">
+    <cfRule type="expression" priority="26" dxfId="0">
+      <formula>ISNUMBER(G11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" priority="27" dxfId="0">
+      <formula>ISNUMBER(H11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A12">
+    <cfRule type="expression" priority="28" dxfId="0">
+      <formula>ISNUMBER(A12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" priority="29" dxfId="0">
+      <formula>OR(B12="Within 1 year",B12="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12">
+    <cfRule type="expression" priority="30" dxfId="0">
+      <formula>ISNUMBER(C12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="expression" priority="31" dxfId="0">
+      <formula>ISNUMBER(D12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12">
+    <cfRule type="expression" priority="32" dxfId="0">
+      <formula>ISNUMBER(E12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12">
+    <cfRule type="expression" priority="33" dxfId="0">
+      <formula>OR(F12="Yes",F12="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12">
+    <cfRule type="expression" priority="34" dxfId="0">
+      <formula>ISNUMBER(G12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" priority="35" dxfId="0">
+      <formula>ISNUMBER(H12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A13">
+    <cfRule type="expression" priority="36" dxfId="0">
+      <formula>ISNUMBER(A13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" priority="37" dxfId="0">
+      <formula>OR(B13="Within 1 year",B13="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="expression" priority="38" dxfId="0">
+      <formula>ISNUMBER(C13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="expression" priority="39" dxfId="0">
+      <formula>ISNUMBER(D13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="expression" priority="40" dxfId="0">
+      <formula>ISNUMBER(E13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F13">
+    <cfRule type="expression" priority="41" dxfId="0">
+      <formula>OR(F13="Yes",F13="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13">
+    <cfRule type="expression" priority="42" dxfId="0">
+      <formula>ISNUMBER(G13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" priority="43" dxfId="0">
+      <formula>ISNUMBER(H13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A14">
+    <cfRule type="expression" priority="44" dxfId="0">
+      <formula>ISNUMBER(A14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" priority="45" dxfId="0">
+      <formula>OR(B14="Within 1 year",B14="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C14">
+    <cfRule type="expression" priority="46" dxfId="0">
+      <formula>ISNUMBER(C14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
+    <cfRule type="expression" priority="47" dxfId="0">
+      <formula>ISNUMBER(D14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14">
+    <cfRule type="expression" priority="48" dxfId="0">
+      <formula>ISNUMBER(E14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F14">
+    <cfRule type="expression" priority="49" dxfId="0">
+      <formula>OR(F14="Yes",F14="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G14">
+    <cfRule type="expression" priority="50" dxfId="0">
+      <formula>ISNUMBER(G14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14">
+    <cfRule type="expression" priority="51" dxfId="0">
+      <formula>ISNUMBER(H14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15">
+    <cfRule type="expression" priority="52" dxfId="0">
+      <formula>ISNUMBER(A15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15">
+    <cfRule type="expression" priority="53" dxfId="0">
+      <formula>OR(B15="Within 1 year",B15="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15">
+    <cfRule type="expression" priority="54" dxfId="0">
+      <formula>ISNUMBER(C15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15">
+    <cfRule type="expression" priority="55" dxfId="0">
+      <formula>ISNUMBER(D15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15">
+    <cfRule type="expression" priority="56" dxfId="0">
+      <formula>ISNUMBER(E15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F15">
+    <cfRule type="expression" priority="57" dxfId="0">
+      <formula>OR(F15="Yes",F15="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
+    <cfRule type="expression" priority="58" dxfId="0">
+      <formula>ISNUMBER(G15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" priority="59" dxfId="0">
+      <formula>ISNUMBER(H15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A16">
+    <cfRule type="expression" priority="60" dxfId="0">
+      <formula>ISNUMBER(A16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16">
+    <cfRule type="expression" priority="61" dxfId="0">
+      <formula>OR(B16="Within 1 year",B16="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16">
+    <cfRule type="expression" priority="62" dxfId="0">
+      <formula>ISNUMBER(C16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16">
+    <cfRule type="expression" priority="63" dxfId="0">
+      <formula>ISNUMBER(D16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="expression" priority="64" dxfId="0">
+      <formula>ISNUMBER(E16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16">
+    <cfRule type="expression" priority="65" dxfId="0">
+      <formula>OR(F16="Yes",F16="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="expression" priority="66" dxfId="0">
+      <formula>ISNUMBER(G16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="expression" priority="67" dxfId="0">
+      <formula>ISNUMBER(H16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A17">
+    <cfRule type="expression" priority="68" dxfId="0">
+      <formula>ISNUMBER(A17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17">
+    <cfRule type="expression" priority="69" dxfId="0">
+      <formula>OR(B17="Within 1 year",B17="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
+    <cfRule type="expression" priority="70" dxfId="0">
+      <formula>ISNUMBER(C17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17">
+    <cfRule type="expression" priority="71" dxfId="0">
+      <formula>ISNUMBER(D17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="expression" priority="72" dxfId="0">
+      <formula>ISNUMBER(E17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17">
+    <cfRule type="expression" priority="73" dxfId="0">
+      <formula>OR(F17="Yes",F17="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
+    <cfRule type="expression" priority="74" dxfId="0">
+      <formula>ISNUMBER(G17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" priority="75" dxfId="0">
+      <formula>ISNUMBER(H17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A18">
+    <cfRule type="expression" priority="76" dxfId="0">
+      <formula>ISNUMBER(A18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="expression" priority="77" dxfId="0">
+      <formula>OR(B18="Within 1 year",B18="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18">
+    <cfRule type="expression" priority="78" dxfId="0">
+      <formula>ISNUMBER(C18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18">
+    <cfRule type="expression" priority="79" dxfId="0">
+      <formula>ISNUMBER(D18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="expression" priority="80" dxfId="0">
+      <formula>ISNUMBER(E18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F18">
+    <cfRule type="expression" priority="81" dxfId="0">
+      <formula>OR(F18="Yes",F18="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
+    <cfRule type="expression" priority="82" dxfId="0">
+      <formula>ISNUMBER(G18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="expression" priority="83" dxfId="0">
+      <formula>ISNUMBER(H18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19">
+    <cfRule type="expression" priority="84" dxfId="0">
+      <formula>ISNUMBER(A19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="expression" priority="85" dxfId="0">
+      <formula>OR(B19="Within 1 year",B19="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19">
+    <cfRule type="expression" priority="86" dxfId="0">
+      <formula>ISNUMBER(C19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19">
+    <cfRule type="expression" priority="87" dxfId="0">
+      <formula>ISNUMBER(D19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="expression" priority="88" dxfId="0">
+      <formula>ISNUMBER(E19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F19">
+    <cfRule type="expression" priority="89" dxfId="0">
+      <formula>OR(F19="Yes",F19="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="expression" priority="90" dxfId="0">
+      <formula>ISNUMBER(G19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="expression" priority="91" dxfId="0">
+      <formula>ISNUMBER(H19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20">
+    <cfRule type="expression" priority="92" dxfId="0">
+      <formula>ISNUMBER(A20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20">
+    <cfRule type="expression" priority="93" dxfId="0">
+      <formula>OR(B20="Within 1 year",B20="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20">
+    <cfRule type="expression" priority="94" dxfId="0">
+      <formula>ISNUMBER(C20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
+    <cfRule type="expression" priority="95" dxfId="0">
+      <formula>ISNUMBER(D20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E20">
+    <cfRule type="expression" priority="96" dxfId="0">
+      <formula>ISNUMBER(E20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F20">
+    <cfRule type="expression" priority="97" dxfId="0">
+      <formula>OR(F20="Yes",F20="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="expression" priority="98" dxfId="0">
+      <formula>ISNUMBER(G20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="expression" priority="99" dxfId="0">
+      <formula>ISNUMBER(H20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="99">
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Rising prices" prompt="How fast prices rise each year. Start with 15%; change it if the latest inflation figure is different."/>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Buffer" prompt="Extra added to every goal for surprises. 10% is a good start."/>
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Monthly saving" prompt="Your monthly surplus: money in minus money out, from your Money Map."/>
+    <dataValidation sqref="A9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
       <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
     </dataValidation>
-    <dataValidation sqref="F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="G9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1218,24 +1927,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>EXAMPLE: Esther's goals</t>
         </is>
       </c>
-      <c r="B1" s="24" t="n"/>
-      <c r="C1" s="24" t="n"/>
-      <c r="D1" s="24" t="n"/>
-      <c r="E1" s="24" t="n"/>
-      <c r="F1" s="24" t="n"/>
-      <c r="G1" s="24" t="n"/>
-      <c r="H1" s="24" t="n"/>
-      <c r="I1" s="24" t="n"/>
-      <c r="J1" s="24" t="n"/>
-      <c r="K1" s="24" t="n"/>
+      <c r="B1" s="29" t="n"/>
+      <c r="C1" s="29" t="n"/>
+      <c r="D1" s="29" t="n"/>
+      <c r="E1" s="29" t="n"/>
+      <c r="F1" s="29" t="n"/>
+      <c r="G1" s="29" t="n"/>
+      <c r="H1" s="29" t="n"/>
+      <c r="I1" s="29" t="n"/>
+      <c r="J1" s="29" t="n"/>
+      <c r="K1" s="29" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>An example to show what a finished planner looks like. Fill in your own on the "My goals" tab.</t>
         </is>
@@ -1277,7 +1986,7 @@
           <t>What I can save each month</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="21" t="n">
         <v>160000</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1344,420 +2053,420 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Starter emergency fund</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Within 1 year</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="21" t="n">
         <v>150000</v>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="21" t="n">
         <v>30000</v>
       </c>
-      <c r="I9" s="15">
-        <f>IF(E9="","",IF(F9="Yes",E9+G9,(E9*(1+$C$4)^C9+G9)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J9" s="15">
-        <f>IF(I9="","",MAX(0,I9-H9))</f>
-        <v/>
-      </c>
-      <c r="K9" s="16">
-        <f>IF(OR(J9="",C9=""),"",IF(C9&lt;=0,J9,J9/(C9*12)))</f>
+      <c r="I9" s="16">
+        <f>IF(NOT(ISNUMBER(E9)),"",IF(F9="Yes",E9+N(G9),(E9*(1+$C$4)^N(C9)+N(G9))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="16">
+        <f>IF(I9="","",MAX(0,I9-N(H9)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="17">
+        <f>IF(OR(J9="",NOT(ISNUMBER(C9))),"",IF(C9&lt;=0,J9,J9/(C9*12)))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Rent (amount agreed with landlord)</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Within 1 year</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="19" t="n">
         <v>0.67</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="21" t="n">
         <v>600000</v>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="21" t="n">
         <v>120000</v>
       </c>
-      <c r="I10" s="15">
-        <f>IF(E10="","",IF(F10="Yes",E10+G10,(E10*(1+$C$4)^C10+G10)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J10" s="15">
-        <f>IF(I10="","",MAX(0,I10-H10))</f>
-        <v/>
-      </c>
-      <c r="K10" s="16">
-        <f>IF(OR(J10="",C10=""),"",IF(C10&lt;=0,J10,J10/(C10*12)))</f>
+      <c r="I10" s="16">
+        <f>IF(NOT(ISNUMBER(E10)),"",IF(F10="Yes",E10+N(G10),(E10*(1+$C$4)^N(C10)+N(G10))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="16">
+        <f>IF(I10="","",MAX(0,I10-N(H10)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="17">
+        <f>IF(OR(J10="",NOT(ISNUMBER(C10))),"",IF(C10&lt;=0,J10,J10/(C10*12)))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Sewing machines for the business</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>1–5 years</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="21" t="n">
         <v>900000</v>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G11" s="21" t="n">
         <v>60000</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="21" t="n">
         <v>200000</v>
       </c>
-      <c r="I11" s="15">
-        <f>IF(E11="","",IF(F11="Yes",E11+G11,(E11*(1+$C$4)^C11+G11)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J11" s="15">
-        <f>IF(I11="","",MAX(0,I11-H11))</f>
-        <v/>
-      </c>
-      <c r="K11" s="16">
-        <f>IF(OR(J11="",C11=""),"",IF(C11&lt;=0,J11,J11/(C11*12)))</f>
+      <c r="I11" s="16">
+        <f>IF(NOT(ISNUMBER(E11)),"",IF(F11="Yes",E11+N(G11),(E11*(1+$C$4)^N(C11)+N(G11))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="16">
+        <f>IF(I11="","",MAX(0,I11-N(H11)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IF(OR(J11="",NOT(ISNUMBER(C11))),"",IF(C11&lt;=0,J11,J11/(C11*12)))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Land deposit</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>5–10 years</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="12" t="n">
+      <c r="D12" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="21" t="n">
         <v>3000000</v>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G12" s="10" t="n">
+      <c r="G12" s="21" t="n">
         <v>250000</v>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="H12" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="15">
-        <f>IF(E12="","",IF(F12="Yes",E12+G12,(E12*(1+$C$4)^C12+G12)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J12" s="15">
-        <f>IF(I12="","",MAX(0,I12-H12))</f>
-        <v/>
-      </c>
-      <c r="K12" s="16">
-        <f>IF(OR(J12="",C12=""),"",IF(C12&lt;=0,J12,J12/(C12*12)))</f>
+      <c r="I12" s="16">
+        <f>IF(NOT(ISNUMBER(E12)),"",IF(F12="Yes",E12+N(G12),(E12*(1+$C$4)^N(C12)+N(G12))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="16">
+        <f>IF(I12="","",MAX(0,I12-N(H12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="17">
+        <f>IF(OR(J12="",NOT(ISNUMBER(C12))),"",IF(C12&lt;=0,J12,J12/(C12*12)))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Children's university (first year)</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>10–20 years</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="21" t="n">
         <v>1000000</v>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="31" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G13" s="10" t="n">
+      <c r="G13" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="10" t="n">
+      <c r="H13" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="15">
-        <f>IF(E13="","",IF(F13="Yes",E13+G13,(E13*(1+$C$4)^C13+G13)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J13" s="15">
-        <f>IF(I13="","",MAX(0,I13-H13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="16">
-        <f>IF(OR(J13="",C13=""),"",IF(C13&lt;=0,J13,J13/(C13*12)))</f>
+      <c r="I13" s="16">
+        <f>IF(NOT(ISNUMBER(E13)),"",IF(F13="Yes",E13+N(G13),(E13*(1+$C$4)^N(C13)+N(G13))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J13" s="16">
+        <f>IF(I13="","",MAX(0,I13-N(H13)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="17">
+        <f>IF(OR(J13="",NOT(ISNUMBER(C13))),"",IF(C13&lt;=0,J13,J13/(C13*12)))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="15">
-        <f>IF(E14="","",IF(F14="Yes",E14+G14,(E14*(1+$C$4)^C14+G14)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J14" s="15">
-        <f>IF(I14="","",MAX(0,I14-H14))</f>
-        <v/>
-      </c>
-      <c r="K14" s="16">
-        <f>IF(OR(J14="",C14=""),"",IF(C14&lt;=0,J14,J14/(C14*12)))</f>
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="13" t="inlineStr"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="13" t="inlineStr"/>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="21" t="n"/>
+      <c r="I14" s="16">
+        <f>IF(NOT(ISNUMBER(E14)),"",IF(F14="Yes",E14+N(G14),(E14*(1+$C$4)^N(C14)+N(G14))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J14" s="16">
+        <f>IF(I14="","",MAX(0,I14-N(H14)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="17">
+        <f>IF(OR(J14="",NOT(ISNUMBER(C14))),"",IF(C14&lt;=0,J14,J14/(C14*12)))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="13" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="10" t="n"/>
-      <c r="I15" s="15">
-        <f>IF(E15="","",IF(F15="Yes",E15+G15,(E15*(1+$C$4)^C15+G15)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J15" s="15">
-        <f>IF(I15="","",MAX(0,I15-H15))</f>
-        <v/>
-      </c>
-      <c r="K15" s="16">
-        <f>IF(OR(J15="",C15=""),"",IF(C15&lt;=0,J15,J15/(C15*12)))</f>
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="13" t="inlineStr"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="13" t="inlineStr"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="16">
+        <f>IF(NOT(ISNUMBER(E15)),"",IF(F15="Yes",E15+N(G15),(E15*(1+$C$4)^N(C15)+N(G15))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J15" s="16">
+        <f>IF(I15="","",MAX(0,I15-N(H15)))</f>
+        <v/>
+      </c>
+      <c r="K15" s="17">
+        <f>IF(OR(J15="",NOT(ISNUMBER(C15))),"",IF(C15&lt;=0,J15,J15/(C15*12)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="13" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="15">
-        <f>IF(E16="","",IF(F16="Yes",E16+G16,(E16*(1+$C$4)^C16+G16)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J16" s="15">
-        <f>IF(I16="","",MAX(0,I16-H16))</f>
-        <v/>
-      </c>
-      <c r="K16" s="16">
-        <f>IF(OR(J16="",C16=""),"",IF(C16&lt;=0,J16,J16/(C16*12)))</f>
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="13" t="inlineStr"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="13" t="inlineStr"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="21" t="n"/>
+      <c r="I16" s="16">
+        <f>IF(NOT(ISNUMBER(E16)),"",IF(F16="Yes",E16+N(G16),(E16*(1+$C$4)^N(C16)+N(G16))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J16" s="16">
+        <f>IF(I16="","",MAX(0,I16-N(H16)))</f>
+        <v/>
+      </c>
+      <c r="K16" s="17">
+        <f>IF(OR(J16="",NOT(ISNUMBER(C16))),"",IF(C16&lt;=0,J16,J16/(C16*12)))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="15">
-        <f>IF(E17="","",IF(F17="Yes",E17+G17,(E17*(1+$C$4)^C17+G17)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J17" s="15">
-        <f>IF(I17="","",MAX(0,I17-H17))</f>
-        <v/>
-      </c>
-      <c r="K17" s="16">
-        <f>IF(OR(J17="",C17=""),"",IF(C17&lt;=0,J17,J17/(C17*12)))</f>
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="13" t="inlineStr"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="16">
+        <f>IF(NOT(ISNUMBER(E17)),"",IF(F17="Yes",E17+N(G17),(E17*(1+$C$4)^N(C17)+N(G17))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J17" s="16">
+        <f>IF(I17="","",MAX(0,I17-N(H17)))</f>
+        <v/>
+      </c>
+      <c r="K17" s="17">
+        <f>IF(OR(J17="",NOT(ISNUMBER(C17))),"",IF(C17&lt;=0,J17,J17/(C17*12)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="13" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="15">
-        <f>IF(E18="","",IF(F18="Yes",E18+G18,(E18*(1+$C$4)^C18+G18)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J18" s="15">
-        <f>IF(I18="","",MAX(0,I18-H18))</f>
-        <v/>
-      </c>
-      <c r="K18" s="16">
-        <f>IF(OR(J18="",C18=""),"",IF(C18&lt;=0,J18,J18/(C18*12)))</f>
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="13" t="inlineStr"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="13" t="inlineStr"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="16">
+        <f>IF(NOT(ISNUMBER(E18)),"",IF(F18="Yes",E18+N(G18),(E18*(1+$C$4)^N(C18)+N(G18))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J18" s="16">
+        <f>IF(I18="","",MAX(0,I18-N(H18)))</f>
+        <v/>
+      </c>
+      <c r="K18" s="17">
+        <f>IF(OR(J18="",NOT(ISNUMBER(C18))),"",IF(C18&lt;=0,J18,J18/(C18*12)))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="15">
-        <f>IF(E19="","",IF(F19="Yes",E19+G19,(E19*(1+$C$4)^C19+G19)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J19" s="15">
-        <f>IF(I19="","",MAX(0,I19-H19))</f>
-        <v/>
-      </c>
-      <c r="K19" s="16">
-        <f>IF(OR(J19="",C19=""),"",IF(C19&lt;=0,J19,J19/(C19*12)))</f>
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="13" t="inlineStr"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="13" t="inlineStr"/>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="16">
+        <f>IF(NOT(ISNUMBER(E19)),"",IF(F19="Yes",E19+N(G19),(E19*(1+$C$4)^N(C19)+N(G19))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J19" s="16">
+        <f>IF(I19="","",MAX(0,I19-N(H19)))</f>
+        <v/>
+      </c>
+      <c r="K19" s="17">
+        <f>IF(OR(J19="",NOT(ISNUMBER(C19))),"",IF(C19&lt;=0,J19,J19/(C19*12)))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="15">
-        <f>IF(E20="","",IF(F20="Yes",E20+G20,(E20*(1+$C$4)^C20+G20)*(1+$C$5)))</f>
-        <v/>
-      </c>
-      <c r="J20" s="15">
-        <f>IF(I20="","",MAX(0,I20-H20))</f>
-        <v/>
-      </c>
-      <c r="K20" s="16">
-        <f>IF(OR(J20="",C20=""),"",IF(C20&lt;=0,J20,J20/(C20*12)))</f>
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="13" t="inlineStr"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="13" t="inlineStr"/>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
+      <c r="I20" s="16">
+        <f>IF(NOT(ISNUMBER(E20)),"",IF(F20="Yes",E20+N(G20),(E20*(1+$C$4)^N(C20)+N(G20))*(1+$C$5)))</f>
+        <v/>
+      </c>
+      <c r="J20" s="16">
+        <f>IF(I20="","",MAX(0,I20-N(H20)))</f>
+        <v/>
+      </c>
+      <c r="K20" s="17">
+        <f>IF(OR(J20="",NOT(ISNUMBER(C20))),"",IF(C20&lt;=0,J20,J20/(C20*12)))</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>Total needed each month for all goals</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n"/>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="n"/>
-      <c r="I22" s="18" t="n"/>
-      <c r="J22" s="18" t="n"/>
-      <c r="K22" s="19">
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="23" t="n"/>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="23" t="n"/>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="23" t="n"/>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="23" t="n"/>
+      <c r="K22" s="24">
         <f>SUM(K9:K20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Can I afford all of them?</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="25" t="inlineStr">
         <is>
           <t>If "Not yet": give each goal a priority, fund the top ones first, move a date later, or start smaller.</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
-      <c r="J23" s="18" t="n"/>
-      <c r="K23" s="17">
-        <f>IF($C$6="","Fill in C6",IF(K22&lt;=$C$6,"Yes","Not yet"))</f>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="23" t="n"/>
+      <c r="J23" s="23" t="n"/>
+      <c r="K23" s="22">
+        <f>IF(NOT(ISNUMBER($C$6)),"Fill in C6",IF(K22&lt;=$C$6,"Yes","Not yet"))</f>
         <v/>
       </c>
     </row>
@@ -1769,27 +2478,663 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Free from the Financial Intelligence class · kopkad.ng/blog. For educational purposes only. This is not financial advice.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>With Snowball, we keep it rolling.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <conditionalFormatting sqref="C4">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(C4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>ISNUMBER(C5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>ISNUMBER(C6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A9">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>ISNUMBER(A9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>OR(B9="Within 1 year",B9="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>ISNUMBER(C9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>ISNUMBER(D9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E9">
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>ISNUMBER(E9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F9">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>OR(F9="Yes",F9="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>ISNUMBER(G9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>ISNUMBER(H9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10">
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>ISNUMBER(A10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>OR(B10="Within 1 year",B10="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
+    <cfRule type="expression" priority="14" dxfId="0">
+      <formula>ISNUMBER(C10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>ISNUMBER(D10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>ISNUMBER(E10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F10">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>OR(F10="Yes",F10="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10">
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>ISNUMBER(G10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>ISNUMBER(H10)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A11">
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>ISNUMBER(A11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>OR(B11="Within 1 year",B11="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
+    <cfRule type="expression" priority="22" dxfId="0">
+      <formula>ISNUMBER(C11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11">
+    <cfRule type="expression" priority="23" dxfId="0">
+      <formula>ISNUMBER(D11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11">
+    <cfRule type="expression" priority="24" dxfId="0">
+      <formula>ISNUMBER(E11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>OR(F11="Yes",F11="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11">
+    <cfRule type="expression" priority="26" dxfId="0">
+      <formula>ISNUMBER(G11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" priority="27" dxfId="0">
+      <formula>ISNUMBER(H11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A12">
+    <cfRule type="expression" priority="28" dxfId="0">
+      <formula>ISNUMBER(A12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" priority="29" dxfId="0">
+      <formula>OR(B12="Within 1 year",B12="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12">
+    <cfRule type="expression" priority="30" dxfId="0">
+      <formula>ISNUMBER(C12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="expression" priority="31" dxfId="0">
+      <formula>ISNUMBER(D12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12">
+    <cfRule type="expression" priority="32" dxfId="0">
+      <formula>ISNUMBER(E12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12">
+    <cfRule type="expression" priority="33" dxfId="0">
+      <formula>OR(F12="Yes",F12="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12">
+    <cfRule type="expression" priority="34" dxfId="0">
+      <formula>ISNUMBER(G12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12">
+    <cfRule type="expression" priority="35" dxfId="0">
+      <formula>ISNUMBER(H12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A13">
+    <cfRule type="expression" priority="36" dxfId="0">
+      <formula>ISNUMBER(A13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" priority="37" dxfId="0">
+      <formula>OR(B13="Within 1 year",B13="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="expression" priority="38" dxfId="0">
+      <formula>ISNUMBER(C13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="expression" priority="39" dxfId="0">
+      <formula>ISNUMBER(D13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13">
+    <cfRule type="expression" priority="40" dxfId="0">
+      <formula>ISNUMBER(E13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F13">
+    <cfRule type="expression" priority="41" dxfId="0">
+      <formula>OR(F13="Yes",F13="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13">
+    <cfRule type="expression" priority="42" dxfId="0">
+      <formula>ISNUMBER(G13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" priority="43" dxfId="0">
+      <formula>ISNUMBER(H13)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A14">
+    <cfRule type="expression" priority="44" dxfId="0">
+      <formula>ISNUMBER(A14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" priority="45" dxfId="0">
+      <formula>OR(B14="Within 1 year",B14="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C14">
+    <cfRule type="expression" priority="46" dxfId="0">
+      <formula>ISNUMBER(C14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
+    <cfRule type="expression" priority="47" dxfId="0">
+      <formula>ISNUMBER(D14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14">
+    <cfRule type="expression" priority="48" dxfId="0">
+      <formula>ISNUMBER(E14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F14">
+    <cfRule type="expression" priority="49" dxfId="0">
+      <formula>OR(F14="Yes",F14="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G14">
+    <cfRule type="expression" priority="50" dxfId="0">
+      <formula>ISNUMBER(G14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H14">
+    <cfRule type="expression" priority="51" dxfId="0">
+      <formula>ISNUMBER(H14)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15">
+    <cfRule type="expression" priority="52" dxfId="0">
+      <formula>ISNUMBER(A15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15">
+    <cfRule type="expression" priority="53" dxfId="0">
+      <formula>OR(B15="Within 1 year",B15="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15">
+    <cfRule type="expression" priority="54" dxfId="0">
+      <formula>ISNUMBER(C15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15">
+    <cfRule type="expression" priority="55" dxfId="0">
+      <formula>ISNUMBER(D15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15">
+    <cfRule type="expression" priority="56" dxfId="0">
+      <formula>ISNUMBER(E15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F15">
+    <cfRule type="expression" priority="57" dxfId="0">
+      <formula>OR(F15="Yes",F15="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
+    <cfRule type="expression" priority="58" dxfId="0">
+      <formula>ISNUMBER(G15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" priority="59" dxfId="0">
+      <formula>ISNUMBER(H15)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A16">
+    <cfRule type="expression" priority="60" dxfId="0">
+      <formula>ISNUMBER(A16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16">
+    <cfRule type="expression" priority="61" dxfId="0">
+      <formula>OR(B16="Within 1 year",B16="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16">
+    <cfRule type="expression" priority="62" dxfId="0">
+      <formula>ISNUMBER(C16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16">
+    <cfRule type="expression" priority="63" dxfId="0">
+      <formula>ISNUMBER(D16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16">
+    <cfRule type="expression" priority="64" dxfId="0">
+      <formula>ISNUMBER(E16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16">
+    <cfRule type="expression" priority="65" dxfId="0">
+      <formula>OR(F16="Yes",F16="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="expression" priority="66" dxfId="0">
+      <formula>ISNUMBER(G16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="expression" priority="67" dxfId="0">
+      <formula>ISNUMBER(H16)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A17">
+    <cfRule type="expression" priority="68" dxfId="0">
+      <formula>ISNUMBER(A17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17">
+    <cfRule type="expression" priority="69" dxfId="0">
+      <formula>OR(B17="Within 1 year",B17="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
+    <cfRule type="expression" priority="70" dxfId="0">
+      <formula>ISNUMBER(C17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17">
+    <cfRule type="expression" priority="71" dxfId="0">
+      <formula>ISNUMBER(D17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17">
+    <cfRule type="expression" priority="72" dxfId="0">
+      <formula>ISNUMBER(E17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17">
+    <cfRule type="expression" priority="73" dxfId="0">
+      <formula>OR(F17="Yes",F17="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
+    <cfRule type="expression" priority="74" dxfId="0">
+      <formula>ISNUMBER(G17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" priority="75" dxfId="0">
+      <formula>ISNUMBER(H17)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A18">
+    <cfRule type="expression" priority="76" dxfId="0">
+      <formula>ISNUMBER(A18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="expression" priority="77" dxfId="0">
+      <formula>OR(B18="Within 1 year",B18="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18">
+    <cfRule type="expression" priority="78" dxfId="0">
+      <formula>ISNUMBER(C18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18">
+    <cfRule type="expression" priority="79" dxfId="0">
+      <formula>ISNUMBER(D18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18">
+    <cfRule type="expression" priority="80" dxfId="0">
+      <formula>ISNUMBER(E18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F18">
+    <cfRule type="expression" priority="81" dxfId="0">
+      <formula>OR(F18="Yes",F18="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
+    <cfRule type="expression" priority="82" dxfId="0">
+      <formula>ISNUMBER(G18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="expression" priority="83" dxfId="0">
+      <formula>ISNUMBER(H18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19">
+    <cfRule type="expression" priority="84" dxfId="0">
+      <formula>ISNUMBER(A19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="expression" priority="85" dxfId="0">
+      <formula>OR(B19="Within 1 year",B19="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19">
+    <cfRule type="expression" priority="86" dxfId="0">
+      <formula>ISNUMBER(C19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19">
+    <cfRule type="expression" priority="87" dxfId="0">
+      <formula>ISNUMBER(D19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="expression" priority="88" dxfId="0">
+      <formula>ISNUMBER(E19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F19">
+    <cfRule type="expression" priority="89" dxfId="0">
+      <formula>OR(F19="Yes",F19="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="expression" priority="90" dxfId="0">
+      <formula>ISNUMBER(G19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="expression" priority="91" dxfId="0">
+      <formula>ISNUMBER(H19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20">
+    <cfRule type="expression" priority="92" dxfId="0">
+      <formula>ISNUMBER(A20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20">
+    <cfRule type="expression" priority="93" dxfId="0">
+      <formula>OR(B20="Within 1 year",B20="20+ years")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20">
+    <cfRule type="expression" priority="94" dxfId="0">
+      <formula>ISNUMBER(C20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
+    <cfRule type="expression" priority="95" dxfId="0">
+      <formula>ISNUMBER(D20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E20">
+    <cfRule type="expression" priority="96" dxfId="0">
+      <formula>ISNUMBER(E20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F20">
+    <cfRule type="expression" priority="97" dxfId="0">
+      <formula>OR(F20="Yes",F20="No")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="expression" priority="98" dxfId="0">
+      <formula>ISNUMBER(G20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="expression" priority="99" dxfId="0">
+      <formula>ISNUMBER(H20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="99">
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Rising prices" prompt="How fast prices rise each year. Start with 15%; change it if the latest inflation figure is different."/>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Buffer" prompt="Extra added to every goal for surprises. 10% is a good start."/>
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Monthly saving" prompt="Your monthly surplus: money in minus money out, from your Money Map."/>
+    <dataValidation sqref="A9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
       <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
     </dataValidation>
-    <dataValidation sqref="F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F9" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="G9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H9" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H11" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H12" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H14" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H15" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H16" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H17" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H18" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H19" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
+    <dataValidation sqref="A20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Goal" prompt="What the goal is, in a few words."/>
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="How far away the goal is." type="list">
+      <formula1>"Within 1 year,1–5 years,5–10 years,10–20 years,20+ years"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Years from now" prompt="How long until you need the money. 6 months = 0.5, 8 months = 0.67, 2 years = 2."/>
+    <dataValidation sqref="D20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Priority" prompt="1 for the goal that comes first. Safety buffer, then expensive debt, then goals by date."/>
+    <dataValidation sqref="E20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Today's price" prompt="What it costs today. Get a real quote if you can."/>
+    <dataValidation sqref="F20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose one of the options in the list." promptTitle="Choose one" prompt="Yes if the price is already agreed for when you need it, like an agreed rent. Then no rising prices or buffer are added." type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Extras" prompt="Delivery, installation, registration, legal or agent fees."/>
+    <dataValidation sqref="H20" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Already saved" prompt="What you have already put aside towards this goal."/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>